<commit_message>
Updated routine - 26 August 2026
</commit_message>
<xml_diff>
--- a/CAP776.xlsx
+++ b/CAP776.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ANISH\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ANISH\OneDrive\Documents\GitHub\daily-routine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589F1FAB-4E70-4960-B6B7-C8A411E27860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAD2E31A-621E-458F-8D94-D5CC2B6E3146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -253,9 +253,6 @@
   </si>
   <si>
     <t>No regular classes. Studied at home and relaxed.</t>
-  </si>
-  <si>
-    <t>Excellent</t>
   </si>
 </sst>
 </file>
@@ -1714,7 +1711,7 @@
         <v>490</v>
       </c>
       <c r="K20" s="16" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="L20" s="16" t="s">
         <v>63</v>

</xml_diff>